<commit_message>
Ajusta planilha de amostras não processadas
</commit_message>
<xml_diff>
--- a/reports/CV/Carga Viral - semana 20 Julho - 26 Julho.xlsx
+++ b/reports/CV/Carga Viral - semana 20 Julho - 26 Julho.xlsx
@@ -644,7 +644,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -926,6 +926,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2183,9 +2186,9 @@
   <sheetData>
     <row r="2"/>
     <row r="3" ht="18" customHeight="1">
-      <c r="B3" s="59" t="inlineStr">
-        <is>
-          <t>Amostras não Processadas (Semana: 13 Julho - 19 Julho)</t>
+      <c r="B3" s="109" t="inlineStr">
+        <is>
+          <t>Amostras não Processadas (Semana: 20 Julho - 26 Julho)</t>
         </is>
       </c>
     </row>
@@ -2205,14 +2208,14 @@
           <t>DATA DE COLHEITA DAS AMOSTRAS</t>
         </is>
       </c>
-      <c r="D5" s="109" t="n"/>
-      <c r="E5" s="109" t="n"/>
-      <c r="F5" s="109" t="n"/>
-      <c r="G5" s="110" t="n"/>
+      <c r="D5" s="110" t="n"/>
+      <c r="E5" s="110" t="n"/>
+      <c r="F5" s="110" t="n"/>
+      <c r="G5" s="111" t="n"/>
     </row>
     <row r="6" ht="33" customHeight="1">
-      <c r="A6" s="111" t="n"/>
-      <c r="B6" s="111" t="n"/>
+      <c r="A6" s="112" t="n"/>
+      <c r="B6" s="112" t="n"/>
       <c r="C6" s="61" t="inlineStr">
         <is>
           <t>&lt;7 dias</t>
@@ -2246,12 +2249,24 @@
           <t>Cabo Delgado</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="B7" s="14" t="n">
+        <v>6121</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>570</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2158</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>1249</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>2117</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>27</v>
+      </c>
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="13" t="n"/>
     </row>
@@ -2261,12 +2276,24 @@
           <t>Carmelo</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
+      <c r="B8" s="14" t="n">
+        <v>732</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>297</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>377</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>36</v>
+      </c>
       <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="n"/>
     </row>
@@ -2276,12 +2303,24 @@
           <t>Chimoio</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="B9" s="14" t="n">
+        <v>5032</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>741</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1728</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>1079</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>1191</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>293</v>
+      </c>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
     </row>
@@ -2291,12 +2330,24 @@
           <t>Dream Beira</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
+      <c r="B10" s="8" t="n">
+        <v>1524</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>853</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>277</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>165</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>74</v>
+      </c>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>
     </row>
@@ -2306,12 +2357,24 @@
           <t>Dream Maputo</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
+      <c r="B11" s="14" t="n">
+        <v>64</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
     </row>
@@ -2321,12 +2384,24 @@
           <t>INS</t>
         </is>
       </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="B12" s="14" t="n">
+        <v>472</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>194</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N12" s="13" t="n"/>
       <c r="O12" s="13" t="n"/>
     </row>
@@ -2336,12 +2411,24 @@
           <t>Lichinga</t>
         </is>
       </c>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
+      <c r="B13" s="14" t="n">
+        <v>435</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>117</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>117</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>158</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>16</v>
+      </c>
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="n"/>
     </row>
@@ -2351,12 +2438,24 @@
           <t>Machava</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="B14" s="14" t="n">
+        <v>1363</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>985</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>195</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>179</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="N14" s="13" t="n"/>
       <c r="O14" s="13" t="n"/>
     </row>
@@ -2366,12 +2465,24 @@
           <t>Mavalane</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
+      <c r="B15" s="8" t="n">
+        <v>955</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>618</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>167</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
     </row>
@@ -2381,12 +2492,24 @@
           <t>Nampula</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
+      <c r="B16" s="8" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>999</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>3268</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>1907</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>2087</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>13</v>
+      </c>
       <c r="N16" s="13" t="n"/>
       <c r="O16" s="13" t="n"/>
     </row>
@@ -2396,12 +2519,24 @@
           <t>Ponta Gea</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
+      <c r="B17" s="8" t="n">
+        <v>4601</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>487</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>1058</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>995</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>2052</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="N17" s="13" t="n"/>
       <c r="O17" s="13" t="n"/>
     </row>
@@ -2411,12 +2546,24 @@
           <t>Quelimane</t>
         </is>
       </c>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
+      <c r="B18" s="14" t="n">
+        <v>2666</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>764</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>929</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>491</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="N18" s="13" t="n"/>
       <c r="O18" s="13" t="n"/>
     </row>
@@ -2426,12 +2573,24 @@
           <t>Tete</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="6" t="n"/>
+      <c r="B19" s="10" t="n">
+        <v>1746</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>923</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>416</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="N19" s="13" t="n"/>
       <c r="O19" s="13" t="n"/>
     </row>
@@ -2441,12 +2600,24 @@
           <t>Xai-Xai</t>
         </is>
       </c>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
+      <c r="B20" s="14" t="n">
+        <v>3428</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>790</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>1878</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>254</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>496</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="O20" s="13" t="n"/>
     </row>
     <row r="21">
@@ -2482,8 +2653,8 @@
       <c r="O21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="111" t="n"/>
-      <c r="B22" s="111" t="n"/>
+      <c r="A22" s="112" t="n"/>
+      <c r="B22" s="112" t="n"/>
       <c r="C22" s="15">
         <f>C21/B21</f>
         <v/>
@@ -2643,33 +2814,33 @@
           <t># Amostras da colheita na US ao registo no Lab</t>
         </is>
       </c>
-      <c r="D3" s="109" t="n"/>
-      <c r="E3" s="109" t="n"/>
-      <c r="F3" s="109" t="n"/>
-      <c r="G3" s="110" t="n"/>
+      <c r="D3" s="110" t="n"/>
+      <c r="E3" s="110" t="n"/>
+      <c r="F3" s="110" t="n"/>
+      <c r="G3" s="111" t="n"/>
       <c r="H3" s="66" t="inlineStr">
         <is>
           <t># Amostras do registo no Lab a análise</t>
         </is>
       </c>
-      <c r="I3" s="109" t="n"/>
-      <c r="J3" s="109" t="n"/>
-      <c r="K3" s="110" t="n"/>
+      <c r="I3" s="110" t="n"/>
+      <c r="J3" s="110" t="n"/>
+      <c r="K3" s="111" t="n"/>
       <c r="L3" s="66" t="inlineStr">
         <is>
           <t># Amostras da analise a validação</t>
         </is>
       </c>
-      <c r="M3" s="109" t="n"/>
-      <c r="N3" s="110" t="n"/>
+      <c r="M3" s="110" t="n"/>
+      <c r="N3" s="111" t="n"/>
       <c r="O3" s="66" t="inlineStr">
         <is>
           <t>Tempo de Resposta Total</t>
         </is>
       </c>
-      <c r="P3" s="109" t="n"/>
-      <c r="Q3" s="109" t="n"/>
-      <c r="R3" s="110" t="n"/>
+      <c r="P3" s="110" t="n"/>
+      <c r="Q3" s="110" t="n"/>
+      <c r="R3" s="111" t="n"/>
       <c r="S3" s="66" t="inlineStr">
         <is>
           <t>TRL (media em dias)</t>
@@ -2680,12 +2851,12 @@
           <t>Incompletude do FSR</t>
         </is>
       </c>
-      <c r="U3" s="109" t="n"/>
-      <c r="V3" s="110" t="n"/>
+      <c r="U3" s="110" t="n"/>
+      <c r="V3" s="111" t="n"/>
     </row>
     <row r="4" ht="28.8" customHeight="1">
-      <c r="A4" s="111" t="n"/>
-      <c r="B4" s="111" t="n"/>
+      <c r="A4" s="112" t="n"/>
+      <c r="B4" s="112" t="n"/>
       <c r="C4" s="66" t="inlineStr">
         <is>
           <t>&lt;7 dias</t>
@@ -2766,7 +2937,7 @@
           <t>&gt;21 dias</t>
         </is>
       </c>
-      <c r="S4" s="111" t="n"/>
+      <c r="S4" s="112" t="n"/>
       <c r="T4" s="66" t="inlineStr">
         <is>
           <t>Sem data de colheita</t>
@@ -3300,23 +3471,23 @@
           <t># Amostras da colheita na US ao registo no Lab</t>
         </is>
       </c>
-      <c r="D24" s="109" t="n"/>
-      <c r="E24" s="109" t="n"/>
-      <c r="F24" s="109" t="n"/>
-      <c r="G24" s="110" t="n"/>
+      <c r="D24" s="110" t="n"/>
+      <c r="E24" s="110" t="n"/>
+      <c r="F24" s="110" t="n"/>
+      <c r="G24" s="111" t="n"/>
       <c r="H24" s="66" t="inlineStr">
         <is>
           <t># Amostras do registo no Lab a análise</t>
         </is>
       </c>
-      <c r="I24" s="109" t="n"/>
-      <c r="J24" s="109" t="n"/>
-      <c r="K24" s="109" t="n"/>
-      <c r="L24" s="110" t="n"/>
+      <c r="I24" s="110" t="n"/>
+      <c r="J24" s="110" t="n"/>
+      <c r="K24" s="110" t="n"/>
+      <c r="L24" s="111" t="n"/>
     </row>
     <row r="25" ht="28.8" customHeight="1">
-      <c r="A25" s="111" t="n"/>
-      <c r="B25" s="111" t="n"/>
+      <c r="A25" s="112" t="n"/>
+      <c r="B25" s="112" t="n"/>
       <c r="C25" s="66" t="inlineStr">
         <is>
           <t>&lt;7 dias</t>
@@ -3860,45 +4031,45 @@
           <t>#Dias da Colheita na US à Recepção no Lab</t>
         </is>
       </c>
-      <c r="L4" s="109" t="n"/>
-      <c r="M4" s="109" t="n"/>
-      <c r="N4" s="109" t="n"/>
-      <c r="O4" s="110" t="n"/>
+      <c r="L4" s="110" t="n"/>
+      <c r="M4" s="110" t="n"/>
+      <c r="N4" s="110" t="n"/>
+      <c r="O4" s="111" t="n"/>
       <c r="P4" s="72" t="inlineStr">
         <is>
           <t>#Dias da Recepção na US ao Registo no Lab</t>
         </is>
       </c>
-      <c r="Q4" s="109" t="n"/>
-      <c r="R4" s="109" t="n"/>
-      <c r="S4" s="109" t="n"/>
-      <c r="T4" s="110" t="n"/>
+      <c r="Q4" s="110" t="n"/>
+      <c r="R4" s="110" t="n"/>
+      <c r="S4" s="110" t="n"/>
+      <c r="T4" s="111" t="n"/>
       <c r="U4" s="72" t="inlineStr">
         <is>
           <t>#Dias do Registo no Lab à Analise</t>
         </is>
       </c>
-      <c r="V4" s="109" t="n"/>
-      <c r="W4" s="109" t="n"/>
-      <c r="X4" s="109" t="n"/>
-      <c r="Y4" s="110" t="n"/>
+      <c r="V4" s="110" t="n"/>
+      <c r="W4" s="110" t="n"/>
+      <c r="X4" s="110" t="n"/>
+      <c r="Y4" s="111" t="n"/>
       <c r="Z4" s="72" t="inlineStr">
         <is>
           <t xml:space="preserve">#Dias da Analise à Validação		</t>
         </is>
       </c>
-      <c r="AA4" s="109" t="n"/>
-      <c r="AB4" s="109" t="n"/>
-      <c r="AC4" s="110" t="n"/>
+      <c r="AA4" s="110" t="n"/>
+      <c r="AB4" s="110" t="n"/>
+      <c r="AC4" s="111" t="n"/>
       <c r="AD4" s="72" t="inlineStr">
         <is>
           <t>Tempo de Resposta Total</t>
         </is>
       </c>
-      <c r="AE4" s="109" t="n"/>
-      <c r="AF4" s="109" t="n"/>
-      <c r="AG4" s="109" t="n"/>
-      <c r="AH4" s="110" t="n"/>
+      <c r="AE4" s="110" t="n"/>
+      <c r="AF4" s="110" t="n"/>
+      <c r="AG4" s="110" t="n"/>
+      <c r="AH4" s="111" t="n"/>
       <c r="AI4" s="72" t="inlineStr">
         <is>
           <t>TRL (dias)</t>
@@ -3906,16 +4077,16 @@
       </c>
     </row>
     <row r="5" ht="29.4" customHeight="1">
-      <c r="A5" s="111" t="n"/>
-      <c r="B5" s="111" t="n"/>
-      <c r="C5" s="111" t="n"/>
-      <c r="D5" s="111" t="n"/>
-      <c r="E5" s="111" t="n"/>
-      <c r="F5" s="111" t="n"/>
-      <c r="G5" s="111" t="n"/>
-      <c r="H5" s="111" t="n"/>
-      <c r="I5" s="111" t="n"/>
-      <c r="J5" s="111" t="n"/>
+      <c r="A5" s="112" t="n"/>
+      <c r="B5" s="112" t="n"/>
+      <c r="C5" s="112" t="n"/>
+      <c r="D5" s="112" t="n"/>
+      <c r="E5" s="112" t="n"/>
+      <c r="F5" s="112" t="n"/>
+      <c r="G5" s="112" t="n"/>
+      <c r="H5" s="112" t="n"/>
+      <c r="I5" s="112" t="n"/>
+      <c r="J5" s="112" t="n"/>
       <c r="K5" s="72" t="inlineStr">
         <is>
           <t>&lt;7 dias</t>
@@ -4036,7 +4207,7 @@
           <t>Sem data de Validação</t>
         </is>
       </c>
-      <c r="AI5" s="111" t="n"/>
+      <c r="AI5" s="112" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -5647,57 +5818,57 @@
           <t>Colheita à Recepção no Disalink</t>
         </is>
       </c>
-      <c r="K4" s="109" t="n"/>
-      <c r="L4" s="109" t="n"/>
-      <c r="M4" s="109" t="n"/>
-      <c r="N4" s="110" t="n"/>
+      <c r="K4" s="110" t="n"/>
+      <c r="L4" s="110" t="n"/>
+      <c r="M4" s="110" t="n"/>
+      <c r="N4" s="111" t="n"/>
       <c r="O4" s="58" t="inlineStr">
         <is>
           <t>Recepção no DisaLink ao Registo no DisaLink</t>
         </is>
       </c>
-      <c r="P4" s="109" t="n"/>
-      <c r="Q4" s="109" t="n"/>
-      <c r="R4" s="109" t="n"/>
-      <c r="S4" s="110" t="n"/>
+      <c r="P4" s="110" t="n"/>
+      <c r="Q4" s="110" t="n"/>
+      <c r="R4" s="110" t="n"/>
+      <c r="S4" s="111" t="n"/>
       <c r="T4" s="58" t="inlineStr">
         <is>
           <t>Registo no DisaLink à Recepção no Lab</t>
         </is>
       </c>
-      <c r="U4" s="109" t="n"/>
-      <c r="V4" s="109" t="n"/>
-      <c r="W4" s="109" t="n"/>
-      <c r="X4" s="110" t="n"/>
+      <c r="U4" s="110" t="n"/>
+      <c r="V4" s="110" t="n"/>
+      <c r="W4" s="110" t="n"/>
+      <c r="X4" s="111" t="n"/>
       <c r="Y4" s="58" t="inlineStr">
         <is>
           <t>Recepção no Lab ao Registo no Lab</t>
         </is>
       </c>
-      <c r="Z4" s="109" t="n"/>
-      <c r="AA4" s="109" t="n"/>
-      <c r="AB4" s="109" t="n"/>
-      <c r="AC4" s="110" t="n"/>
+      <c r="Z4" s="110" t="n"/>
+      <c r="AA4" s="110" t="n"/>
+      <c r="AB4" s="110" t="n"/>
+      <c r="AC4" s="111" t="n"/>
       <c r="AD4" s="58" t="inlineStr">
         <is>
           <t>Colheita à Recepção no Lab</t>
         </is>
       </c>
-      <c r="AE4" s="109" t="n"/>
-      <c r="AF4" s="109" t="n"/>
-      <c r="AG4" s="109" t="n"/>
-      <c r="AH4" s="110" t="n"/>
+      <c r="AE4" s="110" t="n"/>
+      <c r="AF4" s="110" t="n"/>
+      <c r="AG4" s="110" t="n"/>
+      <c r="AH4" s="111" t="n"/>
     </row>
     <row r="5" ht="34.2" customHeight="1">
-      <c r="A5" s="111" t="n"/>
-      <c r="B5" s="111" t="n"/>
-      <c r="C5" s="111" t="n"/>
-      <c r="D5" s="111" t="n"/>
-      <c r="E5" s="111" t="n"/>
-      <c r="F5" s="111" t="n"/>
-      <c r="G5" s="111" t="n"/>
-      <c r="H5" s="111" t="n"/>
-      <c r="I5" s="111" t="n"/>
+      <c r="A5" s="112" t="n"/>
+      <c r="B5" s="112" t="n"/>
+      <c r="C5" s="112" t="n"/>
+      <c r="D5" s="112" t="n"/>
+      <c r="E5" s="112" t="n"/>
+      <c r="F5" s="112" t="n"/>
+      <c r="G5" s="112" t="n"/>
+      <c r="H5" s="112" t="n"/>
+      <c r="I5" s="112" t="n"/>
       <c r="J5" s="58" t="inlineStr">
         <is>
           <t>&lt;7 dias</t>

</xml_diff>

<commit_message>
Updated report generation for Monitoria das Amostras sheet
</commit_message>
<xml_diff>
--- a/reports/CV/Carga Viral - semana 20 Julho - 26 Julho.xlsx
+++ b/reports/CV/Carga Viral - semana 20 Julho - 26 Julho.xlsx
@@ -2960,27 +2960,69 @@
           <t>Cabo Delgado</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="18" t="n"/>
-      <c r="D5" s="18" t="n"/>
-      <c r="E5" s="18" t="n"/>
-      <c r="F5" s="18" t="n"/>
-      <c r="G5" s="18" t="n"/>
-      <c r="H5" s="19" t="n"/>
-      <c r="I5" s="19" t="n"/>
-      <c r="J5" s="19" t="n"/>
-      <c r="K5" s="19" t="n"/>
-      <c r="L5" s="20" t="n"/>
-      <c r="M5" s="20" t="n"/>
-      <c r="N5" s="20" t="n"/>
-      <c r="O5" s="22" t="n"/>
-      <c r="P5" s="22" t="n"/>
-      <c r="Q5" s="22" t="n"/>
-      <c r="R5" s="22" t="n"/>
-      <c r="S5" s="27" t="n"/>
-      <c r="T5" s="23" t="n"/>
-      <c r="U5" s="23" t="n"/>
-      <c r="V5" s="23" t="n"/>
+      <c r="B5" s="21" t="n">
+        <v>1225</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>812</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>324</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="G5" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>658</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>434</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>88</v>
+      </c>
+      <c r="L5" s="20" t="n">
+        <v>1212</v>
+      </c>
+      <c r="M5" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="N5" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="P5" s="22" t="n">
+        <v>229</v>
+      </c>
+      <c r="Q5" s="22" t="n">
+        <v>489</v>
+      </c>
+      <c r="R5" s="22" t="n">
+        <v>472</v>
+      </c>
+      <c r="S5" s="27" t="n">
+        <v>22</v>
+      </c>
+      <c r="T5" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="U5" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="V5" s="23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
@@ -2988,27 +3030,69 @@
           <t>Carmelo</t>
         </is>
       </c>
-      <c r="B6" s="21" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="18" t="n"/>
-      <c r="E6" s="18" t="n"/>
-      <c r="F6" s="18" t="n"/>
-      <c r="G6" s="18" t="n"/>
-      <c r="H6" s="19" t="n"/>
-      <c r="I6" s="19" t="n"/>
-      <c r="J6" s="19" t="n"/>
-      <c r="K6" s="19" t="n"/>
-      <c r="L6" s="20" t="n"/>
-      <c r="M6" s="20" t="n"/>
-      <c r="N6" s="20" t="n"/>
-      <c r="O6" s="22" t="n"/>
-      <c r="P6" s="22" t="n"/>
-      <c r="Q6" s="22" t="n"/>
-      <c r="R6" s="22" t="n"/>
-      <c r="S6" s="27" t="n"/>
-      <c r="T6" s="23" t="n"/>
-      <c r="U6" s="23" t="n"/>
-      <c r="V6" s="23" t="n"/>
+      <c r="B6" s="21" t="n">
+        <v>805</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>485</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>301</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>802</v>
+      </c>
+      <c r="I6" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="20" t="n">
+        <v>558</v>
+      </c>
+      <c r="M6" s="20" t="n">
+        <v>247</v>
+      </c>
+      <c r="N6" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="22" t="n">
+        <v>171</v>
+      </c>
+      <c r="P6" s="22" t="n">
+        <v>604</v>
+      </c>
+      <c r="Q6" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="R6" s="22" t="n">
+        <v>17</v>
+      </c>
+      <c r="S6" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="T6" s="23" t="n">
+        <v>36</v>
+      </c>
+      <c r="U6" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="V6" s="23" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
@@ -3016,27 +3100,69 @@
           <t>Chimoio</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="19" t="n"/>
-      <c r="I7" s="19" t="n"/>
-      <c r="J7" s="19" t="n"/>
-      <c r="K7" s="19" t="n"/>
-      <c r="L7" s="20" t="n"/>
-      <c r="M7" s="20" t="n"/>
-      <c r="N7" s="20" t="n"/>
-      <c r="O7" s="22" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="27" t="n"/>
-      <c r="T7" s="23" t="n"/>
-      <c r="U7" s="23" t="n"/>
-      <c r="V7" s="23" t="n"/>
+      <c r="B7" s="21" t="n">
+        <v>2966</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>2433</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>481</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>1324</v>
+      </c>
+      <c r="I7" s="19" t="n">
+        <v>1391</v>
+      </c>
+      <c r="J7" s="19" t="n">
+        <v>240</v>
+      </c>
+      <c r="K7" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="L7" s="20" t="n">
+        <v>2966</v>
+      </c>
+      <c r="M7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="22" t="n">
+        <v>481</v>
+      </c>
+      <c r="P7" s="22" t="n">
+        <v>1461</v>
+      </c>
+      <c r="Q7" s="22" t="n">
+        <v>826</v>
+      </c>
+      <c r="R7" s="22" t="n">
+        <v>184</v>
+      </c>
+      <c r="S7" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="T7" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="U7" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="V7" s="23" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="30" t="inlineStr">
@@ -3044,27 +3170,69 @@
           <t>Dream Beira</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
-      <c r="G8" s="18" t="n"/>
-      <c r="H8" s="19" t="n"/>
-      <c r="I8" s="19" t="n"/>
-      <c r="J8" s="19" t="n"/>
-      <c r="K8" s="19" t="n"/>
-      <c r="L8" s="20" t="n"/>
-      <c r="M8" s="20" t="n"/>
-      <c r="N8" s="20" t="n"/>
-      <c r="O8" s="22" t="n"/>
-      <c r="P8" s="22" t="n"/>
-      <c r="Q8" s="22" t="n"/>
-      <c r="R8" s="22" t="n"/>
-      <c r="S8" s="27" t="n"/>
-      <c r="T8" s="23" t="n"/>
-      <c r="U8" s="23" t="n"/>
-      <c r="V8" s="23" t="n"/>
+      <c r="B8" s="21" t="n">
+        <v>1694</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>386</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>724</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>349</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>1367</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>325</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="20" t="n">
+        <v>1685</v>
+      </c>
+      <c r="M8" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="N8" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="22" t="n">
+        <v>344</v>
+      </c>
+      <c r="P8" s="22" t="n">
+        <v>526</v>
+      </c>
+      <c r="Q8" s="22" t="n">
+        <v>339</v>
+      </c>
+      <c r="R8" s="22" t="n">
+        <v>450</v>
+      </c>
+      <c r="S8" s="27" t="n">
+        <v>19</v>
+      </c>
+      <c r="T8" s="23" t="n">
+        <v>109</v>
+      </c>
+      <c r="U8" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="V8" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
@@ -3072,27 +3240,69 @@
           <t>Dream Maputo</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="19" t="n"/>
-      <c r="I9" s="19" t="n"/>
-      <c r="J9" s="19" t="n"/>
-      <c r="K9" s="19" t="n"/>
-      <c r="L9" s="20" t="n"/>
-      <c r="M9" s="20" t="n"/>
-      <c r="N9" s="20" t="n"/>
-      <c r="O9" s="22" t="n"/>
-      <c r="P9" s="22" t="n"/>
-      <c r="Q9" s="22" t="n"/>
-      <c r="R9" s="22" t="n"/>
-      <c r="S9" s="27" t="n"/>
-      <c r="T9" s="23" t="n"/>
-      <c r="U9" s="23" t="n"/>
-      <c r="V9" s="23" t="n"/>
+      <c r="B9" s="21" t="n">
+        <v>741</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>740</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>741</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="20" t="n">
+        <v>453</v>
+      </c>
+      <c r="M9" s="20" t="n">
+        <v>288</v>
+      </c>
+      <c r="N9" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="22" t="n">
+        <v>680</v>
+      </c>
+      <c r="P9" s="22" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="T9" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="V9" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
@@ -3100,27 +3310,69 @@
           <t>INS</t>
         </is>
       </c>
-      <c r="B10" s="21" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="18" t="n"/>
-      <c r="F10" s="18" t="n"/>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="19" t="n"/>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="20" t="n"/>
-      <c r="M10" s="20" t="n"/>
-      <c r="N10" s="20" t="n"/>
-      <c r="O10" s="22" t="n"/>
-      <c r="P10" s="22" t="n"/>
-      <c r="Q10" s="22" t="n"/>
-      <c r="R10" s="22" t="n"/>
-      <c r="S10" s="27" t="n"/>
-      <c r="T10" s="23" t="n"/>
-      <c r="U10" s="23" t="n"/>
-      <c r="V10" s="23" t="n"/>
+      <c r="B10" s="21" t="n">
+        <v>621</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>333</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>154</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>450</v>
+      </c>
+      <c r="I10" s="19" t="n">
+        <v>170</v>
+      </c>
+      <c r="J10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="20" t="n">
+        <v>620</v>
+      </c>
+      <c r="M10" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="22" t="n">
+        <v>37</v>
+      </c>
+      <c r="P10" s="22" t="n">
+        <v>371</v>
+      </c>
+      <c r="Q10" s="22" t="n">
+        <v>86</v>
+      </c>
+      <c r="R10" s="22" t="n">
+        <v>123</v>
+      </c>
+      <c r="S10" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="T10" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="23" t="n">
+        <v>0</v>
+      </c>
       <c r="X10" s="13" t="n"/>
       <c r="Y10" s="13" t="n"/>
       <c r="Z10" s="13" t="n"/>
@@ -3131,27 +3383,69 @@
           <t>Lichinga</t>
         </is>
       </c>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
-      <c r="J11" s="19" t="n"/>
-      <c r="K11" s="19" t="n"/>
-      <c r="L11" s="20" t="n"/>
-      <c r="M11" s="20" t="n"/>
-      <c r="N11" s="20" t="n"/>
-      <c r="O11" s="22" t="n"/>
-      <c r="P11" s="22" t="n"/>
-      <c r="Q11" s="22" t="n"/>
-      <c r="R11" s="22" t="n"/>
-      <c r="S11" s="27" t="n"/>
-      <c r="T11" s="23" t="n"/>
-      <c r="U11" s="23" t="n"/>
-      <c r="V11" s="23" t="n"/>
+      <c r="B11" s="21" t="n">
+        <v>853</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>486</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>275</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>37</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="G11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>853</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="20" t="n">
+        <v>802</v>
+      </c>
+      <c r="M11" s="20" t="n">
+        <v>51</v>
+      </c>
+      <c r="N11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="22" t="n">
+        <v>317</v>
+      </c>
+      <c r="P11" s="22" t="n">
+        <v>423</v>
+      </c>
+      <c r="Q11" s="22" t="n">
+        <v>52</v>
+      </c>
+      <c r="R11" s="22" t="n">
+        <v>60</v>
+      </c>
+      <c r="S11" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="T11" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="U11" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="V11" s="23" t="n">
+        <v>3</v>
+      </c>
       <c r="X11" s="13" t="n"/>
       <c r="Y11" s="13" t="n"/>
       <c r="Z11" s="13" t="n"/>
@@ -3162,27 +3456,69 @@
           <t>Machava</t>
         </is>
       </c>
-      <c r="B12" s="21" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="18" t="n"/>
-      <c r="F12" s="18" t="n"/>
-      <c r="G12" s="18" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
-      <c r="J12" s="19" t="n"/>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="20" t="n"/>
-      <c r="M12" s="20" t="n"/>
-      <c r="N12" s="20" t="n"/>
-      <c r="O12" s="22" t="n"/>
-      <c r="P12" s="22" t="n"/>
-      <c r="Q12" s="22" t="n"/>
-      <c r="R12" s="22" t="n"/>
-      <c r="S12" s="27" t="n"/>
-      <c r="T12" s="38" t="n"/>
-      <c r="U12" s="38" t="n"/>
-      <c r="V12" s="38" t="n"/>
+      <c r="B12" s="21" t="n">
+        <v>734</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>604</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>124</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>705</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>29</v>
+      </c>
+      <c r="J12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="20" t="n">
+        <v>734</v>
+      </c>
+      <c r="M12" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="22" t="n">
+        <v>462</v>
+      </c>
+      <c r="P12" s="22" t="n">
+        <v>234</v>
+      </c>
+      <c r="Q12" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="R12" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="S12" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="T12" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="U12" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="V12" s="38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="30" t="inlineStr">
@@ -3190,27 +3526,69 @@
           <t>Mavalane</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="18" t="n"/>
-      <c r="E13" s="18" t="n"/>
-      <c r="F13" s="18" t="n"/>
-      <c r="G13" s="18" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
-      <c r="J13" s="19" t="n"/>
-      <c r="K13" s="19" t="n"/>
-      <c r="L13" s="20" t="n"/>
-      <c r="M13" s="20" t="n"/>
-      <c r="N13" s="20" t="n"/>
-      <c r="O13" s="22" t="n"/>
-      <c r="P13" s="22" t="n"/>
-      <c r="Q13" s="22" t="n"/>
-      <c r="R13" s="22" t="n"/>
-      <c r="S13" s="27" t="n"/>
-      <c r="T13" s="38" t="n"/>
-      <c r="U13" s="38" t="n"/>
-      <c r="V13" s="38" t="n"/>
+      <c r="B13" s="21" t="n">
+        <v>3990</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>3891</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>84</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>2746</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>1190</v>
+      </c>
+      <c r="J13" s="19" t="n">
+        <v>36</v>
+      </c>
+      <c r="K13" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="L13" s="20" t="n">
+        <v>3990</v>
+      </c>
+      <c r="M13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="22" t="n">
+        <v>1842</v>
+      </c>
+      <c r="P13" s="22" t="n">
+        <v>2067</v>
+      </c>
+      <c r="Q13" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="R13" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="S13" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="T13" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="U13" s="38" t="n">
+        <v>16</v>
+      </c>
+      <c r="V13" s="38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
@@ -3218,27 +3596,69 @@
           <t>Nampula</t>
         </is>
       </c>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
-      <c r="E14" s="18" t="n"/>
-      <c r="F14" s="18" t="n"/>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="19" t="n"/>
-      <c r="I14" s="19" t="n"/>
-      <c r="J14" s="19" t="n"/>
-      <c r="K14" s="19" t="n"/>
-      <c r="L14" s="20" t="n"/>
-      <c r="M14" s="20" t="n"/>
-      <c r="N14" s="20" t="n"/>
-      <c r="O14" s="22" t="n"/>
-      <c r="P14" s="22" t="n"/>
-      <c r="Q14" s="22" t="n"/>
-      <c r="R14" s="22" t="n"/>
-      <c r="S14" s="27" t="n"/>
-      <c r="T14" s="38" t="n"/>
-      <c r="U14" s="38" t="n"/>
-      <c r="V14" s="38" t="n"/>
+      <c r="B14" s="21" t="n">
+        <v>6218</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>3050</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>2206</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>522</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>424</v>
+      </c>
+      <c r="G14" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>122</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>2835</v>
+      </c>
+      <c r="J14" s="19" t="n">
+        <v>2574</v>
+      </c>
+      <c r="K14" s="19" t="n">
+        <v>687</v>
+      </c>
+      <c r="L14" s="20" t="n">
+        <v>3696</v>
+      </c>
+      <c r="M14" s="20" t="n">
+        <v>2521</v>
+      </c>
+      <c r="N14" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" s="22" t="n">
+        <v>319</v>
+      </c>
+      <c r="Q14" s="22" t="n">
+        <v>1631</v>
+      </c>
+      <c r="R14" s="22" t="n">
+        <v>4245</v>
+      </c>
+      <c r="S14" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="T14" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="U14" s="38" t="n">
+        <v>47</v>
+      </c>
+      <c r="V14" s="38" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="30" t="inlineStr">
@@ -3246,27 +3666,69 @@
           <t>Ponta Gea</t>
         </is>
       </c>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="19" t="n"/>
-      <c r="I15" s="19" t="n"/>
-      <c r="J15" s="19" t="n"/>
-      <c r="K15" s="19" t="n"/>
-      <c r="L15" s="20" t="n"/>
-      <c r="M15" s="20" t="n"/>
-      <c r="N15" s="20" t="n"/>
-      <c r="O15" s="22" t="n"/>
-      <c r="P15" s="22" t="n"/>
-      <c r="Q15" s="22" t="n"/>
-      <c r="R15" s="22" t="n"/>
-      <c r="S15" s="27" t="n"/>
-      <c r="T15" s="23" t="n"/>
-      <c r="U15" s="23" t="n"/>
-      <c r="V15" s="23" t="n"/>
+      <c r="B15" s="21" t="n">
+        <v>3882</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>1707</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>1795</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>225</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>144</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>1179</v>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>444</v>
+      </c>
+      <c r="J15" s="19" t="n">
+        <v>263</v>
+      </c>
+      <c r="K15" s="19" t="n">
+        <v>1996</v>
+      </c>
+      <c r="L15" s="20" t="n">
+        <v>3852</v>
+      </c>
+      <c r="M15" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="N15" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="22" t="n">
+        <v>669</v>
+      </c>
+      <c r="P15" s="22" t="n">
+        <v>531</v>
+      </c>
+      <c r="Q15" s="22" t="n">
+        <v>276</v>
+      </c>
+      <c r="R15" s="22" t="n">
+        <v>2395</v>
+      </c>
+      <c r="S15" s="27" t="n">
+        <v>34</v>
+      </c>
+      <c r="T15" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="U15" s="23" t="n">
+        <v>31</v>
+      </c>
+      <c r="V15" s="23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
@@ -3274,27 +3736,69 @@
           <t>Quelimane</t>
         </is>
       </c>
-      <c r="B16" s="21" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="19" t="n"/>
-      <c r="I16" s="19" t="n"/>
-      <c r="J16" s="19" t="n"/>
-      <c r="K16" s="19" t="n"/>
-      <c r="L16" s="20" t="n"/>
-      <c r="M16" s="20" t="n"/>
-      <c r="N16" s="20" t="n"/>
-      <c r="O16" s="22" t="n"/>
-      <c r="P16" s="22" t="n"/>
-      <c r="Q16" s="22" t="n"/>
-      <c r="R16" s="22" t="n"/>
-      <c r="S16" s="27" t="n"/>
-      <c r="T16" s="23" t="n"/>
-      <c r="U16" s="23" t="n"/>
-      <c r="V16" s="23" t="n"/>
+      <c r="B16" s="21" t="n">
+        <v>8135</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>5168</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>2129</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>245</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>532</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>61</v>
+      </c>
+      <c r="H16" s="19" t="n">
+        <v>7923</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>189</v>
+      </c>
+      <c r="J16" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="K16" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="L16" s="20" t="n">
+        <v>8133</v>
+      </c>
+      <c r="M16" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="22" t="n">
+        <v>3080</v>
+      </c>
+      <c r="P16" s="22" t="n">
+        <v>3776</v>
+      </c>
+      <c r="Q16" s="22" t="n">
+        <v>589</v>
+      </c>
+      <c r="R16" s="22" t="n">
+        <v>629</v>
+      </c>
+      <c r="S16" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="T16" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="U16" s="23" t="n">
+        <v>34</v>
+      </c>
+      <c r="V16" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -3302,27 +3806,69 @@
           <t>Tete</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="19" t="n"/>
-      <c r="I17" s="19" t="n"/>
-      <c r="J17" s="19" t="n"/>
-      <c r="K17" s="19" t="n"/>
-      <c r="L17" s="20" t="n"/>
-      <c r="M17" s="20" t="n"/>
-      <c r="N17" s="20" t="n"/>
-      <c r="O17" s="22" t="n"/>
-      <c r="P17" s="22" t="n"/>
-      <c r="Q17" s="22" t="n"/>
-      <c r="R17" s="22" t="n"/>
-      <c r="S17" s="27" t="n"/>
-      <c r="T17" s="23" t="n"/>
-      <c r="U17" s="23" t="n"/>
-      <c r="V17" s="23" t="n"/>
+      <c r="B17" s="21" t="n">
+        <v>1651</v>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>370</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>719</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>195</v>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>351</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="H17" s="19" t="n">
+        <v>1426</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>224</v>
+      </c>
+      <c r="J17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="20" t="n">
+        <v>1544</v>
+      </c>
+      <c r="M17" s="20" t="n">
+        <v>107</v>
+      </c>
+      <c r="N17" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="22" t="n">
+        <v>114</v>
+      </c>
+      <c r="P17" s="22" t="n">
+        <v>777</v>
+      </c>
+      <c r="Q17" s="22" t="n">
+        <v>275</v>
+      </c>
+      <c r="R17" s="22" t="n">
+        <v>469</v>
+      </c>
+      <c r="S17" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="T17" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="U17" s="23" t="n">
+        <v>51</v>
+      </c>
+      <c r="V17" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -3330,27 +3876,69 @@
           <t>Xai-Xai</t>
         </is>
       </c>
-      <c r="B18" s="21" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="19" t="n"/>
-      <c r="I18" s="19" t="n"/>
-      <c r="J18" s="19" t="n"/>
-      <c r="K18" s="19" t="n"/>
-      <c r="L18" s="20" t="n"/>
-      <c r="M18" s="20" t="n"/>
-      <c r="N18" s="20" t="n"/>
-      <c r="O18" s="22" t="n"/>
-      <c r="P18" s="22" t="n"/>
-      <c r="Q18" s="22" t="n"/>
-      <c r="R18" s="22" t="n"/>
-      <c r="S18" s="27" t="n"/>
-      <c r="T18" s="23" t="n"/>
-      <c r="U18" s="23" t="n"/>
-      <c r="V18" s="23" t="n"/>
+      <c r="B18" s="21" t="n">
+        <v>6696</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>2512</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>1547</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>195</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>2425</v>
+      </c>
+      <c r="G18" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>6553</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>141</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="20" t="n">
+        <v>6318</v>
+      </c>
+      <c r="M18" s="20" t="n">
+        <v>378</v>
+      </c>
+      <c r="N18" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="22" t="n">
+        <v>917</v>
+      </c>
+      <c r="P18" s="22" t="n">
+        <v>2964</v>
+      </c>
+      <c r="Q18" s="22" t="n">
+        <v>294</v>
+      </c>
+      <c r="R18" s="22" t="n">
+        <v>2504</v>
+      </c>
+      <c r="S18" s="27" t="n">
+        <v>21</v>
+      </c>
+      <c r="T18" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="U18" s="23" t="n">
+        <v>62</v>
+      </c>
+      <c r="V18" s="23" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" customFormat="1" s="5">
       <c r="A19" s="31" t="inlineStr">

</xml_diff>